<commit_message>
AC1 - widen verificationOutcome to serve AcceptanceCheck
The three existing entries each gain a second Occurrence for
//diggs:AcceptanceCheck/diggs:outcome, so a design-side and an as-built verdict read
the same way rather than through parallel vocabularies. This is the R11/PR3 move: an
existing vocabulary made usable in a new context instead of a new one invented.

Adds waived - the requirement was not met and the departure was accepted rather than
corrected. Distinct from not_satisfied, which records a failure without saying what
followed, and from not_required, which means the requirement never applied. Pairs
with NonConformance/disposition = accept_as_is.

waived is bound to AcceptanceCheck only: a design verification is satisfied, not
satisfied, or not required, and there is no party to grant a concession against a
calculation.

23 additions, 0 deletions - the quote-escaping artifact did not fire here.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/verificationOutcome.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/verificationOutcome.xlsx
@@ -1170,12 +1170,32 @@
         <f>IF(ISNA(VLOOKUP(B5,AssociatedElements!B$2:B2943,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B5" s="13" t="n"/>
-      <c r="C5" s="13" t="n"/>
-      <c r="D5" s="14" t="n"/>
-      <c r="E5" s="13" t="n"/>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>waived</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Waived</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>The requirement was not met, and the departure was accepted rather than corrected - the outcome of a formal concession. Distinguished from not_satisfied, which records a failure without saying what followed, and from not_required, which means the requirement never applied to this subject in the first place. A waived check should normally cite, through nonConformanceRef, the diggs:NonConformance whose disposition records the concession; the pairing is with the accept_as_is disposition. Bound to diggs:AcceptanceCheck only: a design verification is either satisfied, not satisfied, or not required, and there is no party to grant a concession against a calculation.</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F5" s="13" t="n"/>
-      <c r="G5" s="9" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2">
@@ -1635,28 +1655,64 @@
         <f>IF(ISNA(VLOOKUP(B5,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B5" s="2" t="n"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>satisfied</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>//diggs:AcceptanceCheck/diggs:outcome</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
         <f>IF(ISNA(VLOOKUP(B6,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B6" s="2" t="n"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>not_satisfied</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>//diggs:AcceptanceCheck/diggs:outcome</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
         <f>IF(ISNA(VLOOKUP(B7,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B7" s="2" t="n"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>not_required</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>//diggs:AcceptanceCheck/diggs:outcome</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
         <f>IF(ISNA(VLOOKUP(B8,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B8" s="2" t="n"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>waived</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>//diggs:AcceptanceCheck/diggs:outcome</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9">

</xml_diff>